<commit_message>
feat(finanzas): proveedores, cuentas y bancos en lote; solo los importados bloquean el mes (099 escrita)
- Documentos existentes: Proveedores y cuentas de los gastos (proveedor por gasto,
  cuenta por linea) y Bancos de los cobros, en lote, admin y contador. Solo
  documentos sin asiento, reales y desde el inicio; uno con asiento no se toca
  (409 sin escribir). Bitacora contable con el usuario.
- Boton Corregir en cada problema del mes.
- Un solo metodo: bloquean solo los asientos importados; los manuales se listan en
  Asientos manuales del mes (pantalla y Excel). 099: la misma regla en la base y
  el banco de un cobro con asiento no cambia.
- Verificacion 097 con los casos 4, 4b y 10 (099). Datos de prueba de staging.
- Consulta de solo lectura: los 5 borradores de produccion.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finanzas/posteo-retroactivo/en-seco-2026-09-01_2026-09-30.xlsx
+++ b/docs/finanzas/posteo-retroactivo/en-seco-2026-09-01_2026-09-30.xlsx
@@ -8,13 +8,15 @@
     <sheet name="Totales por cuenta" sheetId="3" r:id="rId3"/>
     <sheet name="No se contabilizan" sheetId="4" r:id="rId4"/>
     <sheet name="Con problemas" sheetId="5" r:id="rId5"/>
+    <sheet name="Asientos manuales del mes" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Léame'!A1:B28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Asientos'!A3:J12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Totales por cuenta'!A1:E7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Léame'!A1:B32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Asientos'!A3:J28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Totales por cuenta'!A1:E9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3">'No se contabilizan'!A1:D8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4">'Con problemas'!A1:D1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'Asientos manuales del mes'!A1:D6</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -412,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B32"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="70.83203125" customWidth="1"/>
@@ -457,126 +459,155 @@
         <v>Asientos</v>
       </c>
       <c r="B7" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Factura</v>
+        <v>Gasto de trámite</v>
       </c>
       <c r="B8" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Nota de crédito</v>
+        <v>Cobro</v>
       </c>
       <c r="B9" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Total débitos</v>
-      </c>
-      <c r="B10" s="2">
-        <v>2257</v>
+        <v>Factura</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Total créditos</v>
-      </c>
-      <c r="B11" s="2">
-        <v>2257</v>
+        <v>Nota de crédito</v>
+      </c>
+      <c r="B11" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>¿Cuadra?</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Sí: débitos = créditos.</v>
+        <v>Total débitos</v>
+      </c>
+      <c r="B12" s="2">
+        <v>2623.75</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>No se contabilizan (a propósito)</v>
-      </c>
-      <c r="B13" s="1">
-        <v>7</v>
+        <v>Total créditos</v>
+      </c>
+      <c r="B13" s="2">
+        <v>2623.75</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Con problemas (hay que corregirlos antes)</v>
-      </c>
-      <c r="B14" s="1">
-        <v>0</v>
+        <v>¿Cuadra?</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Sí: débitos = créditos.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>No se contabilizan (a propósito)</v>
+      </c>
+      <c r="B15" s="1">
+        <v>7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Cómo leer las hojas</v>
+        <v>Con problemas (hay que corregirlos antes)</v>
+      </c>
+      <c r="B16" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Asientos: una fila por línea de cada asiento, en orden de fecha. Débito y crédito en balboas.</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Totales por cuenta: lo que el período movería en cada cuenta.</v>
+        <v>Asientos manuales del mes (revisar)</v>
+      </c>
+      <c r="B17" s="1">
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>No se contabilizan: documentos que quedan fuera a propósito, con el motivo.</v>
+        <v>Cómo leer las hojas</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Con problemas: documentos que no se pueden registrar hasta corregirlos (por ejemplo, un gasto sin proveedor o un cobro sin banco).</v>
+        <v>Asientos: una fila por línea de cada asiento, en orden de fecha. Débito y crédito en balboas.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Totales por cuenta: lo que el período movería en cada cuenta.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Antes de contabilizar</v>
+        <v>No se contabilizan: documentos que quedan fuera a propósito, con el motivo.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>• El período ya tiene 5 asiento(s) manuales o importados: asiento 88 (30/09/2026, adelanto de efectivo); asiento 15 (10/09/2026, Depreciacion de mobiliario — verificacion 10/09); PRUEBA-75 (25/09/2026, Prueba 7.5: provisión de sueldos de septiembre); asiento 19 (11/09/2026, prueba); asiento 87 (25/09/2026, Prueba 7.5: combustible pagado con banco). Un mes se carga por un solo método: no se contabilizan los documentos.</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>Avisos</v>
+        <v>Con problemas: documentos que no se pueden registrar hasta corregirlos (por ejemplo, un gasto sin proveedor o un cobro sin banco).</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Asientos manuales del mes: los ajustes cargados a mano en el período. No impiden contabilizar. Revisa que ninguno registre un documento que también está en la hoja Asientos.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
+        <v>Antes de contabilizar</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>• El período ya tiene 2 asiento(s) importados: PRUEBA-75 (25/09/2026, Prueba 7.5: provisión de sueldos de septiembre); asiento 87 (25/09/2026, Prueba 7.5: combustible pagado con banco). Un mes se carga por un solo método: no se contabilizan los documentos.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Avisos</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
         <v>• FAC-HON-000007 (04/09/2026) no tiene CUFE en el CRM y SÍ se contabiliza.</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Generado el 10/07/2026, 3:24:01 p. m.</v>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Generado el 10/07/2026, 3:59:46 p. m.</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B28"/>
+  <autoFilter ref="A1:B32"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B32"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J28"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -632,28 +663,28 @@
         <v>1</v>
       </c>
       <c r="B4" t="str">
-        <v>Factura</v>
+        <v>Gasto de trámite</v>
       </c>
       <c r="C4" t="str">
-        <v>FAC-HON-000007</v>
+        <v>PRUEBA-LOTE-G1 (N.º FAC-CO- se asigna al contabilizar)</v>
       </c>
       <c r="D4" s="3">
-        <v>46269</v>
+        <v>46267</v>
       </c>
       <c r="E4" t="str">
-        <v>Aurelio Barría Quintero (CLI-009)</v>
+        <v>CABLE ONDA S.A (PRV-001)</v>
       </c>
       <c r="F4" t="str">
-        <v>100004</v>
+        <v>130003</v>
       </c>
       <c r="G4" t="str">
-        <v>Cuentas por Cobrar Clientes</v>
+        <v>Fondo Legales de Clientes</v>
       </c>
       <c r="H4" t="str">
-        <v>Factura FAC-HON-000007</v>
+        <v>Certificación registral</v>
       </c>
       <c r="I4" s="2">
-        <v>107</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -661,57 +692,57 @@
         <v>1</v>
       </c>
       <c r="B5" t="str">
-        <v>Factura</v>
+        <v>Gasto de trámite</v>
       </c>
       <c r="C5" t="str">
-        <v>FAC-HON-000007</v>
+        <v>PRUEBA-LOTE-G1 (N.º FAC-CO- se asigna al contabilizar)</v>
       </c>
       <c r="D5" s="3">
-        <v>46269</v>
+        <v>46267</v>
       </c>
       <c r="E5" t="str">
-        <v>Aurelio Barría Quintero (CLI-009)</v>
+        <v>CABLE ONDA S.A (PRV-001)</v>
       </c>
       <c r="F5" t="str">
-        <v>400004</v>
+        <v>200001</v>
       </c>
       <c r="G5" t="str">
-        <v>Derecho Civil</v>
+        <v>Cuentas por pagar</v>
       </c>
       <c r="H5" t="str">
-        <v>Honorarios civiles</v>
+        <v>CABLE ONDA S.A</v>
       </c>
       <c r="J5" s="2">
-        <v>100</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B6" t="str">
-        <v>Factura</v>
+        <v>Cobro</v>
       </c>
       <c r="C6" t="str">
-        <v>FAC-HON-000007</v>
+        <v>CO-920001</v>
       </c>
       <c r="D6" s="3">
-        <v>46269</v>
+        <v>46268</v>
       </c>
       <c r="E6" t="str">
-        <v>Aurelio Barría Quintero (CLI-009)</v>
+        <v>FERRETERÍA VALLARINO, S.A. (CLI-001)</v>
       </c>
       <c r="F6" t="str">
-        <v>200003</v>
+        <v>100001</v>
       </c>
       <c r="G6" t="str">
-        <v>ITBMS por Pagar</v>
+        <v>Banco General Operativa</v>
       </c>
       <c r="H6" t="str">
-        <v>ITBMS facturado</v>
-      </c>
-      <c r="J6" s="2">
-        <v>7</v>
+        <v>Cobro sin aplicar</v>
+      </c>
+      <c r="I6" s="2">
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -719,16 +750,16 @@
         <v>2</v>
       </c>
       <c r="B7" t="str">
-        <v>Nota de crédito</v>
+        <v>Cobro</v>
       </c>
       <c r="C7" t="str">
-        <v>NC-000010</v>
+        <v>CO-920001</v>
       </c>
       <c r="D7" s="3">
-        <v>46289</v>
+        <v>46268</v>
       </c>
       <c r="E7" t="str">
-        <v>CONSTRUCTORA CHIRIQUÍ ANTIGUO, S.A. (CLI-005)</v>
+        <v>FERRETERÍA VALLARINO, S.A. (CLI-001)</v>
       </c>
       <c r="F7" t="str">
         <v>100004</v>
@@ -737,39 +768,39 @@
         <v>Cuentas por Cobrar Clientes</v>
       </c>
       <c r="H7" t="str">
-        <v>Nota de crédito NC-000010, factura FAC-REI-000004</v>
+        <v>FERRETERÍA VALLARINO, S.A.</v>
       </c>
       <c r="J7" s="2">
-        <v>10</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B8" t="str">
-        <v>Nota de crédito</v>
+        <v>Factura</v>
       </c>
       <c r="C8" t="str">
-        <v>NC-000010</v>
+        <v>FAC-HON-000007</v>
       </c>
       <c r="D8" s="3">
-        <v>46289</v>
+        <v>46269</v>
       </c>
       <c r="E8" t="str">
-        <v>CONSTRUCTORA CHIRIQUÍ ANTIGUO, S.A. (CLI-005)</v>
+        <v>Aurelio Barría Quintero (CLI-009)</v>
       </c>
       <c r="F8" t="str">
-        <v>130003</v>
+        <v>100004</v>
       </c>
       <c r="G8" t="str">
-        <v>Fondo Legales de Clientes</v>
+        <v>Cuentas por Cobrar Clientes</v>
       </c>
       <c r="H8" t="str">
-        <v>Prueba 9B — medir la respuesta de la anulación ante la DGI</v>
+        <v>Factura FAC-HON-000007</v>
       </c>
       <c r="I8" s="2">
-        <v>10</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9">
@@ -777,28 +808,28 @@
         <v>3</v>
       </c>
       <c r="B9" t="str">
-        <v>Nota de crédito</v>
+        <v>Factura</v>
       </c>
       <c r="C9" t="str">
-        <v>NC-000012</v>
+        <v>FAC-HON-000007</v>
       </c>
       <c r="D9" s="3">
-        <v>46289</v>
+        <v>46269</v>
       </c>
       <c r="E9" t="str">
-        <v>PANAMÁ COSTA VERDE, S.A. (CLI-002)</v>
+        <v>Aurelio Barría Quintero (CLI-009)</v>
       </c>
       <c r="F9" t="str">
-        <v>100004</v>
+        <v>400004</v>
       </c>
       <c r="G9" t="str">
-        <v>Cuentas por Cobrar Clientes</v>
+        <v>Derecho Civil</v>
       </c>
       <c r="H9" t="str">
-        <v>Nota de crédito NC-000012, factura FAC-HON-000003</v>
+        <v>Honorarios civiles</v>
       </c>
       <c r="J9" s="2">
-        <v>2140</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
@@ -806,81 +837,545 @@
         <v>3</v>
       </c>
       <c r="B10" t="str">
-        <v>Nota de crédito</v>
+        <v>Factura</v>
       </c>
       <c r="C10" t="str">
-        <v>NC-000012</v>
+        <v>FAC-HON-000007</v>
       </c>
       <c r="D10" s="3">
-        <v>46289</v>
+        <v>46269</v>
       </c>
       <c r="E10" t="str">
-        <v>PANAMÁ COSTA VERDE, S.A. (CLI-002)</v>
+        <v>Aurelio Barría Quintero (CLI-009)</v>
       </c>
       <c r="F10" t="str">
-        <v>400010</v>
+        <v>200003</v>
       </c>
       <c r="G10" t="str">
-        <v>Otros servicios</v>
+        <v>ITBMS por Pagar</v>
       </c>
       <c r="H10" t="str">
-        <v>Honorarios — recurso de reconsideración</v>
-      </c>
-      <c r="I10" s="2">
-        <v>2000</v>
+        <v>ITBMS facturado</v>
+      </c>
+      <c r="J10" s="2">
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B11" t="str">
+        <v>Gasto de trámite</v>
+      </c>
+      <c r="C11" t="str">
+        <v>PRUEBA-LOTE-G2 (N.º FAC-CO- se asigna al contabilizar)</v>
+      </c>
+      <c r="D11" s="3">
+        <v>46269</v>
+      </c>
+      <c r="E11" t="str">
+        <v>CABLE ONDA S.A (PRV-001)</v>
+      </c>
+      <c r="F11" t="str">
+        <v>130003</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Fondo Legales de Clientes</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Timbres fiscales</v>
+      </c>
+      <c r="I11" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1">
+        <v>4</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Gasto de trámite</v>
+      </c>
+      <c r="C12" t="str">
+        <v>PRUEBA-LOTE-G2 (N.º FAC-CO- se asigna al contabilizar)</v>
+      </c>
+      <c r="D12" s="3">
+        <v>46269</v>
+      </c>
+      <c r="E12" t="str">
+        <v>CABLE ONDA S.A (PRV-001)</v>
+      </c>
+      <c r="F12" t="str">
+        <v>130003</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Fondo Legales de Clientes</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Copias autenticadas</v>
+      </c>
+      <c r="I12" s="2">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1">
+        <v>4</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Gasto de trámite</v>
+      </c>
+      <c r="C13" t="str">
+        <v>PRUEBA-LOTE-G2 (N.º FAC-CO- se asigna al contabilizar)</v>
+      </c>
+      <c r="D13" s="3">
+        <v>46269</v>
+      </c>
+      <c r="E13" t="str">
+        <v>CABLE ONDA S.A (PRV-001)</v>
+      </c>
+      <c r="F13" t="str">
+        <v>200001</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Cuentas por pagar</v>
+      </c>
+      <c r="H13" t="str">
+        <v>CABLE ONDA S.A</v>
+      </c>
+      <c r="J13" s="2">
+        <v>20.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1">
+        <v>5</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Gasto de trámite</v>
+      </c>
+      <c r="C14" t="str">
+        <v>PRUEBA-LOTE-G3 (N.º FAC-CO- se asigna al contabilizar)</v>
+      </c>
+      <c r="D14" s="3">
+        <v>46273</v>
+      </c>
+      <c r="E14" t="str">
+        <v>CABLE ONDA S.A (PRV-001)</v>
+      </c>
+      <c r="F14" t="str">
+        <v>130003</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Fondo Legales de Clientes</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Tasa de inscripción</v>
+      </c>
+      <c r="I14" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1">
+        <v>5</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Gasto de trámite</v>
+      </c>
+      <c r="C15" t="str">
+        <v>PRUEBA-LOTE-G3 (N.º FAC-CO- se asigna al contabilizar)</v>
+      </c>
+      <c r="D15" s="3">
+        <v>46273</v>
+      </c>
+      <c r="E15" t="str">
+        <v>CABLE ONDA S.A (PRV-001)</v>
+      </c>
+      <c r="F15" t="str">
+        <v>130003</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Fondo Legales de Clientes</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Mensajería</v>
+      </c>
+      <c r="I15" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1">
+        <v>5</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Gasto de trámite</v>
+      </c>
+      <c r="C16" t="str">
+        <v>PRUEBA-LOTE-G3 (N.º FAC-CO- se asigna al contabilizar)</v>
+      </c>
+      <c r="D16" s="3">
+        <v>46273</v>
+      </c>
+      <c r="E16" t="str">
+        <v>CABLE ONDA S.A (PRV-001)</v>
+      </c>
+      <c r="F16" t="str">
+        <v>200001</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Cuentas por pagar</v>
+      </c>
+      <c r="H16" t="str">
+        <v>CABLE ONDA S.A</v>
+      </c>
+      <c r="J16" s="2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1">
+        <v>6</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Cobro</v>
+      </c>
+      <c r="C17" t="str">
+        <v>CO-920002</v>
+      </c>
+      <c r="D17" s="3">
+        <v>46275</v>
+      </c>
+      <c r="E17" t="str">
+        <v>FERRETERÍA VALLARINO, S.A. (CLI-001)</v>
+      </c>
+      <c r="F17" t="str">
+        <v>100001</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Banco General Operativa</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Cobro sin aplicar</v>
+      </c>
+      <c r="I17" s="2">
+        <v>75.25</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1">
+        <v>6</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Cobro</v>
+      </c>
+      <c r="C18" t="str">
+        <v>CO-920002</v>
+      </c>
+      <c r="D18" s="3">
+        <v>46275</v>
+      </c>
+      <c r="E18" t="str">
+        <v>FERRETERÍA VALLARINO, S.A. (CLI-001)</v>
+      </c>
+      <c r="F18" t="str">
+        <v>100004</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Cuentas por Cobrar Clientes</v>
+      </c>
+      <c r="H18" t="str">
+        <v>FERRETERÍA VALLARINO, S.A.</v>
+      </c>
+      <c r="J18" s="2">
+        <v>75.25</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1">
+        <v>7</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Gasto de trámite</v>
+      </c>
+      <c r="C19" t="str">
+        <v>PRUEBA-LOTE-G4 (N.º FAC-CO- se asigna al contabilizar)</v>
+      </c>
+      <c r="D19" s="3">
+        <v>46276</v>
+      </c>
+      <c r="E19" t="str">
+        <v>CABLE ONDA S.A (PRV-001)</v>
+      </c>
+      <c r="F19" t="str">
+        <v>130003</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Fondo Legales de Clientes</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Notaría: autenticación de firmas</v>
+      </c>
+      <c r="I19" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1">
+        <v>7</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Gasto de trámite</v>
+      </c>
+      <c r="C20" t="str">
+        <v>PRUEBA-LOTE-G4 (N.º FAC-CO- se asigna al contabilizar)</v>
+      </c>
+      <c r="D20" s="3">
+        <v>46276</v>
+      </c>
+      <c r="E20" t="str">
+        <v>CABLE ONDA S.A (PRV-001)</v>
+      </c>
+      <c r="F20" t="str">
+        <v>200001</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Cuentas por pagar</v>
+      </c>
+      <c r="H20" t="str">
+        <v>CABLE ONDA S.A</v>
+      </c>
+      <c r="J20" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1">
+        <v>8</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Cobro</v>
+      </c>
+      <c r="C21" t="str">
+        <v>CO-920003</v>
+      </c>
+      <c r="D21" s="3">
+        <v>46280</v>
+      </c>
+      <c r="E21" t="str">
+        <v>FERRETERÍA VALLARINO, S.A. (CLI-001)</v>
+      </c>
+      <c r="F21" t="str">
+        <v>100001</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Banco General Operativa</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Cobro sin aplicar</v>
+      </c>
+      <c r="I21" s="2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1">
+        <v>8</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Cobro</v>
+      </c>
+      <c r="C22" t="str">
+        <v>CO-920003</v>
+      </c>
+      <c r="D22" s="3">
+        <v>46280</v>
+      </c>
+      <c r="E22" t="str">
+        <v>FERRETERÍA VALLARINO, S.A. (CLI-001)</v>
+      </c>
+      <c r="F22" t="str">
+        <v>100004</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Cuentas por Cobrar Clientes</v>
+      </c>
+      <c r="H22" t="str">
+        <v>FERRETERÍA VALLARINO, S.A.</v>
+      </c>
+      <c r="J22" s="2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1">
+        <v>9</v>
+      </c>
+      <c r="B23" t="str">
         <v>Nota de crédito</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C23" t="str">
+        <v>NC-000010</v>
+      </c>
+      <c r="D23" s="3">
+        <v>46289</v>
+      </c>
+      <c r="E23" t="str">
+        <v>CONSTRUCTORA CHIRIQUÍ ANTIGUO, S.A. (CLI-005)</v>
+      </c>
+      <c r="F23" t="str">
+        <v>100004</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Cuentas por Cobrar Clientes</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Nota de crédito NC-000010, factura FAC-REI-000004</v>
+      </c>
+      <c r="J23" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1">
+        <v>9</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Nota de crédito</v>
+      </c>
+      <c r="C24" t="str">
+        <v>NC-000010</v>
+      </c>
+      <c r="D24" s="3">
+        <v>46289</v>
+      </c>
+      <c r="E24" t="str">
+        <v>CONSTRUCTORA CHIRIQUÍ ANTIGUO, S.A. (CLI-005)</v>
+      </c>
+      <c r="F24" t="str">
+        <v>130003</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Fondo Legales de Clientes</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Prueba 9B — medir la respuesta de la anulación ante la DGI</v>
+      </c>
+      <c r="I24" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1">
+        <v>10</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Nota de crédito</v>
+      </c>
+      <c r="C25" t="str">
         <v>NC-000012</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D25" s="3">
         <v>46289</v>
       </c>
-      <c r="E11" t="str">
+      <c r="E25" t="str">
         <v>PANAMÁ COSTA VERDE, S.A. (CLI-002)</v>
       </c>
-      <c r="F11" t="str">
+      <c r="F25" t="str">
+        <v>100004</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Cuentas por Cobrar Clientes</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Nota de crédito NC-000012, factura FAC-HON-000003</v>
+      </c>
+      <c r="J25" s="2">
+        <v>2140</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1">
+        <v>10</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Nota de crédito</v>
+      </c>
+      <c r="C26" t="str">
+        <v>NC-000012</v>
+      </c>
+      <c r="D26" s="3">
+        <v>46289</v>
+      </c>
+      <c r="E26" t="str">
+        <v>PANAMÁ COSTA VERDE, S.A. (CLI-002)</v>
+      </c>
+      <c r="F26" t="str">
+        <v>400010</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Otros servicios</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Honorarios — recurso de reconsideración</v>
+      </c>
+      <c r="I26" s="2">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1">
+        <v>10</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Nota de crédito</v>
+      </c>
+      <c r="C27" t="str">
+        <v>NC-000012</v>
+      </c>
+      <c r="D27" s="3">
+        <v>46289</v>
+      </c>
+      <c r="E27" t="str">
+        <v>PANAMÁ COSTA VERDE, S.A. (CLI-002)</v>
+      </c>
+      <c r="F27" t="str">
         <v>200003</v>
       </c>
-      <c r="G11" t="str">
+      <c r="G27" t="str">
         <v>ITBMS por Pagar</v>
       </c>
-      <c r="H11" t="str">
+      <c r="H27" t="str">
         <v>ITBMS acreditado</v>
       </c>
-      <c r="I11" s="2">
+      <c r="I27" s="2">
         <v>140</v>
       </c>
     </row>
-    <row r="12">
-      <c r="H12" t="str">
+    <row r="28">
+      <c r="H28" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="I12" s="2">
-        <v>2257</v>
-      </c>
-      <c r="J12" s="2">
-        <v>2257</v>
+      <c r="I28" s="2">
+        <v>2623.75</v>
+      </c>
+      <c r="J28" s="2">
+        <v>2623.75</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J12"/>
+  <autoFilter ref="A3:J28"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J28"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="36.83203125" customWidth="1"/>
@@ -908,107 +1403,141 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>100004</v>
+        <v>100001</v>
       </c>
       <c r="B2" t="str">
-        <v>Cuentas por Cobrar Clientes</v>
+        <v>Banco General Operativa</v>
       </c>
       <c r="C2" s="2">
-        <v>107</v>
+        <v>245.25</v>
       </c>
       <c r="D2" s="2">
-        <v>2150</v>
+        <v>0</v>
       </c>
       <c r="E2" s="2">
-        <v>-2043</v>
+        <v>245.25</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>130003</v>
+        <v>100004</v>
       </c>
       <c r="B3" t="str">
-        <v>Fondo Legales de Clientes</v>
+        <v>Cuentas por Cobrar Clientes</v>
       </c>
       <c r="C3" s="2">
-        <v>10</v>
+        <v>107</v>
       </c>
       <c r="D3" s="2">
-        <v>0</v>
+        <v>2395.25</v>
       </c>
       <c r="E3" s="2">
-        <v>10</v>
+        <v>-2288.25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>200003</v>
+        <v>130003</v>
       </c>
       <c r="B4" t="str">
-        <v>ITBMS por Pagar</v>
+        <v>Fondo Legales de Clientes</v>
       </c>
       <c r="C4" s="2">
-        <v>140</v>
+        <v>131.5</v>
       </c>
       <c r="D4" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E4" s="2">
-        <v>133</v>
+        <v>131.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>400004</v>
+        <v>200001</v>
       </c>
       <c r="B5" t="str">
-        <v>Derecho Civil</v>
+        <v>Cuentas por pagar</v>
       </c>
       <c r="C5" s="2">
         <v>0</v>
       </c>
       <c r="D5" s="2">
-        <v>100</v>
+        <v>121.5</v>
       </c>
       <c r="E5" s="2">
-        <v>-100</v>
+        <v>-121.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>400010</v>
+        <v>200003</v>
       </c>
       <c r="B6" t="str">
-        <v>Otros servicios</v>
+        <v>ITBMS por Pagar</v>
       </c>
       <c r="C6" s="2">
-        <v>2000</v>
+        <v>140</v>
       </c>
       <c r="D6" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E6" s="2">
-        <v>2000</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>400004</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Derecho Civil</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0</v>
+      </c>
+      <c r="D7" s="2">
+        <v>100</v>
+      </c>
+      <c r="E7" s="2">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>400010</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Otros servicios</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2000</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="C7" s="2">
-        <v>2257</v>
-      </c>
-      <c r="D7" s="2">
-        <v>2257</v>
-      </c>
-      <c r="E7" s="2">
+      <c r="C9" s="2">
+        <v>2623.75</v>
+      </c>
+      <c r="D9" s="2">
+        <v>2623.75</v>
+      </c>
+      <c r="E9" s="2">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:E9"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1173,4 +1702,83 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D6"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Número</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Fecha</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Descripción</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Monto</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Revisa que ninguno registre un documento que también está en la hoja Asientos.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>asiento 15</v>
+      </c>
+      <c r="B4" s="3">
+        <v>46275</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Depreciacion de mobiliario — verificacion 10/09</v>
+      </c>
+      <c r="D4" s="2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>asiento 19</v>
+      </c>
+      <c r="B5" s="3">
+        <v>46276</v>
+      </c>
+      <c r="C5" t="str">
+        <v>prueba</v>
+      </c>
+      <c r="D5" s="2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>asiento 88</v>
+      </c>
+      <c r="B6" s="3">
+        <v>46295</v>
+      </c>
+      <c r="C6" t="str">
+        <v>adelanto de efectivo</v>
+      </c>
+      <c r="D6" s="2">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D6"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>